<commit_message>
feat(dashboards): larger membership sample counts with more drop offs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HOL Final Feature list QA 30-Oct-2026 Design Links.xlsx
+++ b/HOL Final Feature list QA 30-Oct-2026 Design Links.xlsx
@@ -18552,9 +18552,9 @@
       <c r="J5" s="87" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="94" t="inlineStr">
-        <is>
-          <t>Not Req</t>
+      <c r="K5" s="148" t="inlineStr">
+        <is>
+          <t>Prototype Link</t>
         </is>
       </c>
       <c r="L5" s="87" t="n"/>
@@ -18640,9 +18640,9 @@
       </c>
       <c r="I7" s="106" t="n"/>
       <c r="J7" s="106" t="n"/>
-      <c r="K7" s="94" t="inlineStr">
-        <is>
-          <t>Not Req</t>
+      <c r="K7" s="148" t="inlineStr">
+        <is>
+          <t>Prototype Link</t>
         </is>
       </c>
       <c r="L7" s="87" t="n"/>
@@ -24542,105 +24542,107 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K141" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K142" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K143" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K144" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K141" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K142" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K143" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K144" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9"/>

</xml_diff>